<commit_message>
✨ feat: created additinal fields kbe and knp
</commit_message>
<xml_diff>
--- a/apps/excel-service/templates/XANSHA/Tax Invoice.xlsx
+++ b/apps/excel-service/templates/XANSHA/Tax Invoice.xlsx
@@ -121,10 +121,42 @@
     <t xml:space="preserve">(ИИН, наименование и адрес)</t>
   </si>
   <si>
-    <t xml:space="preserve">Грузополучатель: {organization.organization}</t>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Грузополучатель: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t>{organization.organization}</t>
+    </r>
   </si>
   <si>
-    <t xml:space="preserve">БИН и адрес места нахождения получателя: БИН:{organization.bin}, {organization.address}</t>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">БИН и адрес места нахождения получателя: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">БИН:{organization.bin}, {organization.address}</t>
+    </r>
   </si>
   <si>
     <r>
@@ -143,7 +175,7 @@
         <color theme="1"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve"> {organization.iik}, {organization.bank}, БИК:{organization.bik} КБЕ: {organization.kbe} КНП: </t>
+      <t xml:space="preserve"> {organization.iik}, {organization.bank}, БИК:{organization.bik} КБЕ: {organization.kbe} </t>
     </r>
     <r>
       <rPr>

</xml_diff>